<commit_message>
feat: Added image extraction tool feature
</commit_message>
<xml_diff>
--- a/server/dataset/Social-Science/Class-8/History/ch8/ch8_descriptions_with_urls.xlsx
+++ b/server/dataset/Social-Science/Class-8/History/ch8/ch8_descriptions_with_urls.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\NCAHT\vision-text_v1.1\server\dataset\Social-Science\Class-8\History\ch8\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92A87C0F-4DCD-4AD4-B544-3E772B166592}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="107">
   <si>
     <t>image-name</t>
   </si>
@@ -134,69 +140,6 @@
   </si>
   <si>
     <t>The Making of the National Movement: 1870s-–1947</t>
-  </si>
-  <si>
-    <t>The Making of the National Movement: 1870s-–1948</t>
-  </si>
-  <si>
-    <t>The Making of the National Movement: 1870s-–1949</t>
-  </si>
-  <si>
-    <t>The Making of the National Movement: 1870s-–1950</t>
-  </si>
-  <si>
-    <t>The Making of the National Movement: 1870s-–1951</t>
-  </si>
-  <si>
-    <t>The Making of the National Movement: 1870s-–1952</t>
-  </si>
-  <si>
-    <t>The Making of the National Movement: 1870s-–1953</t>
-  </si>
-  <si>
-    <t>The Making of the National Movement: 1870s-–1954</t>
-  </si>
-  <si>
-    <t>The Making of the National Movement: 1870s-–1955</t>
-  </si>
-  <si>
-    <t>The Making of the National Movement: 1870s-–1956</t>
-  </si>
-  <si>
-    <t>The Making of the National Movement: 1870s-–1957</t>
-  </si>
-  <si>
-    <t>The Making of the National Movement: 1870s-–1958</t>
-  </si>
-  <si>
-    <t>The Making of the National Movement: 1870s-–1959</t>
-  </si>
-  <si>
-    <t>The Making of the National Movement: 1870s-–1960</t>
-  </si>
-  <si>
-    <t>The Making of the National Movement: 1870s-–1961</t>
-  </si>
-  <si>
-    <t>The Making of the National Movement: 1870s-–1962</t>
-  </si>
-  <si>
-    <t>The Making of the National Movement: 1870s-–1963</t>
-  </si>
-  <si>
-    <t>The Making of the National Movement: 1870s-–1964</t>
-  </si>
-  <si>
-    <t>The Making of the National Movement: 1870s-–1965</t>
-  </si>
-  <si>
-    <t>The Making of the National Movement: 1870s-–1966</t>
-  </si>
-  <si>
-    <t>The Making of the National Movement: 1870s-–1967</t>
-  </si>
-  <si>
-    <t>The Making of the National Movement: 1870s-–1968</t>
   </si>
   <si>
     <t>History</t>
@@ -429,8 +372,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -452,6 +395,12 @@
       <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -506,13 +455,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -550,7 +507,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -584,6 +541,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -618,9 +576,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -793,11 +752,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K23"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="6" max="6" width="47.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -832,7 +794,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -852,19 +814,19 @@
         <v>39</v>
       </c>
       <c r="H2" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="I2" t="s">
-        <v>62</v>
+        <v>41</v>
       </c>
       <c r="J2" t="s">
-        <v>84</v>
+        <v>63</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -881,22 +843,22 @@
         <v>8</v>
       </c>
       <c r="F3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H3" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="I3" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="J3" t="s">
-        <v>85</v>
+        <v>64</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -913,22 +875,22 @@
         <v>8</v>
       </c>
       <c r="F4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="H4" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="I4" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
       <c r="J4" t="s">
-        <v>86</v>
+        <v>65</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -945,22 +907,22 @@
         <v>8</v>
       </c>
       <c r="F5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="H5" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="I5" t="s">
-        <v>65</v>
+        <v>44</v>
       </c>
       <c r="J5" t="s">
-        <v>87</v>
+        <v>66</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -977,22 +939,22 @@
         <v>8</v>
       </c>
       <c r="F6" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="H6" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="I6" t="s">
-        <v>66</v>
+        <v>45</v>
       </c>
       <c r="J6" t="s">
-        <v>88</v>
+        <v>67</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -1009,22 +971,22 @@
         <v>8</v>
       </c>
       <c r="F7" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="H7" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="I7" t="s">
-        <v>67</v>
+        <v>46</v>
       </c>
       <c r="J7" t="s">
-        <v>89</v>
+        <v>68</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -1041,22 +1003,22 @@
         <v>8</v>
       </c>
       <c r="F8" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="H8" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="I8" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="J8" t="s">
-        <v>90</v>
+        <v>69</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -1073,22 +1035,22 @@
         <v>8</v>
       </c>
       <c r="F9" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="H9" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="I9" t="s">
-        <v>69</v>
+        <v>48</v>
       </c>
       <c r="J9" t="s">
-        <v>91</v>
+        <v>70</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -1105,22 +1067,22 @@
         <v>8</v>
       </c>
       <c r="F10" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="H10" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="I10" t="s">
-        <v>70</v>
+        <v>49</v>
       </c>
       <c r="J10" t="s">
-        <v>92</v>
+        <v>71</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -1137,22 +1099,22 @@
         <v>8</v>
       </c>
       <c r="F11" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="H11" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="I11" t="s">
-        <v>71</v>
+        <v>50</v>
       </c>
       <c r="J11" t="s">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -1169,22 +1131,22 @@
         <v>8</v>
       </c>
       <c r="F12" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="H12" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="I12" t="s">
-        <v>72</v>
+        <v>51</v>
       </c>
       <c r="J12" t="s">
-        <v>94</v>
+        <v>73</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -1201,22 +1163,22 @@
         <v>8</v>
       </c>
       <c r="F13" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="H13" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="I13" t="s">
-        <v>73</v>
+        <v>52</v>
       </c>
       <c r="J13" t="s">
-        <v>95</v>
+        <v>74</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -1233,22 +1195,22 @@
         <v>8</v>
       </c>
       <c r="F14" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="H14" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="I14" t="s">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="J14" t="s">
-        <v>96</v>
+        <v>75</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>24</v>
       </c>
@@ -1265,22 +1227,22 @@
         <v>8</v>
       </c>
       <c r="F15" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="H15" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="I15" t="s">
-        <v>75</v>
+        <v>54</v>
       </c>
       <c r="J15" t="s">
-        <v>97</v>
+        <v>76</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>25</v>
       </c>
@@ -1297,22 +1259,22 @@
         <v>8</v>
       </c>
       <c r="F16" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="H16" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="I16" t="s">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="J16" t="s">
-        <v>98</v>
+        <v>77</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>26</v>
       </c>
@@ -1329,22 +1291,22 @@
         <v>8</v>
       </c>
       <c r="F17" t="s">
-        <v>54</v>
+        <v>39</v>
       </c>
       <c r="H17" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="I17" t="s">
-        <v>77</v>
+        <v>56</v>
       </c>
       <c r="J17" t="s">
-        <v>99</v>
+        <v>78</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>27</v>
       </c>
@@ -1361,22 +1323,22 @@
         <v>8</v>
       </c>
       <c r="F18" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="H18" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="I18" t="s">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="J18" t="s">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>28</v>
       </c>
@@ -1393,22 +1355,22 @@
         <v>8</v>
       </c>
       <c r="F19" t="s">
-        <v>56</v>
+        <v>39</v>
       </c>
       <c r="H19" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="I19" t="s">
-        <v>79</v>
+        <v>58</v>
       </c>
       <c r="J19" t="s">
-        <v>101</v>
+        <v>80</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>29</v>
       </c>
@@ -1425,22 +1387,22 @@
         <v>8</v>
       </c>
       <c r="F20" t="s">
-        <v>57</v>
+        <v>39</v>
       </c>
       <c r="H20" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="I20" t="s">
-        <v>80</v>
+        <v>59</v>
       </c>
       <c r="J20" t="s">
-        <v>102</v>
+        <v>81</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>30</v>
       </c>
@@ -1457,22 +1419,22 @@
         <v>8</v>
       </c>
       <c r="F21" t="s">
-        <v>58</v>
+        <v>39</v>
       </c>
       <c r="H21" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="I21" t="s">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="J21" t="s">
-        <v>103</v>
+        <v>82</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>31</v>
       </c>
@@ -1489,22 +1451,22 @@
         <v>8</v>
       </c>
       <c r="F22" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="H22" t="s">
+        <v>40</v>
+      </c>
+      <c r="I22" t="s">
         <v>61</v>
       </c>
-      <c r="I22" t="s">
-        <v>82</v>
-      </c>
       <c r="J22" t="s">
-        <v>104</v>
+        <v>83</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>32</v>
       </c>
@@ -1521,45 +1483,46 @@
         <v>8</v>
       </c>
       <c r="F23" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="H23" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="I23" t="s">
-        <v>83</v>
+        <v>62</v>
       </c>
       <c r="J23" t="s">
-        <v>105</v>
+        <v>84</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>127</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="K2" r:id="rId1"/>
-    <hyperlink ref="K3" r:id="rId2"/>
-    <hyperlink ref="K4" r:id="rId3"/>
-    <hyperlink ref="K5" r:id="rId4"/>
-    <hyperlink ref="K6" r:id="rId5"/>
-    <hyperlink ref="K7" r:id="rId6"/>
-    <hyperlink ref="K8" r:id="rId7"/>
-    <hyperlink ref="K9" r:id="rId8"/>
-    <hyperlink ref="K10" r:id="rId9"/>
-    <hyperlink ref="K11" r:id="rId10"/>
-    <hyperlink ref="K12" r:id="rId11"/>
-    <hyperlink ref="K13" r:id="rId12"/>
-    <hyperlink ref="K14" r:id="rId13"/>
-    <hyperlink ref="K15" r:id="rId14"/>
-    <hyperlink ref="K16" r:id="rId15"/>
-    <hyperlink ref="K17" r:id="rId16"/>
-    <hyperlink ref="K18" r:id="rId17"/>
-    <hyperlink ref="K19" r:id="rId18"/>
-    <hyperlink ref="K20" r:id="rId19"/>
-    <hyperlink ref="K21" r:id="rId20"/>
-    <hyperlink ref="K22" r:id="rId21"/>
-    <hyperlink ref="K23" r:id="rId22"/>
+    <hyperlink ref="K2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="K3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="K4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="K5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="K6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="K7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="K8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="K9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="K10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="K11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="K12" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="K13" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="K14" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="K15" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="K16" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="K17" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="K18" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="K19" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="K20" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="K21" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="K22" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="K23" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>